<commit_message>
feat: complete every workshop task, including the manual ones
- Ruler-style measurements (scripts/p4_medidas_perfiles.py): median brightness
  profiles along both axes, edge at 10 % of the peak-to-sky contrast (5 % and
  20 % as sensitivity), no 2-D smoothing; agree with the automatic method
  within 8 % for AKARI and Planck 857, and match RC3 and SIMBAD for the optical
  LMC and 30 Doradus, where the 3-sigma method misses the faint halo
- Aladin Desktop captures via SAMP with the rulers drawn, Mellinger RGB,
  Bonanos stars and NGC 4755 labelled; SIMBAD page capture
- Fix the Excel chart (invisible markers, B-V axis drawn on top), verified by
  rendering it with LibreOffice
- Worksheet estimates written onto the photo of page 2
- Answers for workshop points 1-3 with SIMBAD cross-checks
- aladin_send: skip SAMP clients that leave the hub mid-call (new test)
</commit_message>
<xml_diff>
--- a/resultados/punto4/Bonanos2009_LMC_V_BV.xlsx
+++ b/resultados/punto4/Bonanos2009_LMC_V_BV.xlsx
@@ -163,7 +163,13 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4FBF"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4FBF"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -186,6 +192,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="3"/>
+          <min val="-1"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -208,11 +216,15 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <crosses val="max"/>
+        <majorUnit val="0.5"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="maxMin"/>
+          <max val="20"/>
+          <min val="9"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -235,11 +247,9 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="min"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>

</xml_diff>